<commit_message>
Egypt/Sharm: RSDC follow-ups answered (sites, eLearning, half board, transfers, hold to end Oct); workbook updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/sharm_group_budget.xlsx
+++ b/december-plan/pricing/sharm_group_budget.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="107">
   <si>
     <t xml:space="preserve">Sharm group budget — inputs (blue cells are editable; USD)</t>
   </si>
@@ -93,28 +93,37 @@
     <t xml:space="preserve">programme</t>
   </si>
   <si>
-    <t xml:space="preserve">PADI Open Water, eLearning done at home: course incl. eLearning registration, full gear, certification</t>
+    <t xml:space="preserve">PADI Open Water: course incl. the PADI eLearning code, full gear, certification</t>
   </si>
   <si>
     <t xml:space="preserve">USD</t>
   </si>
   <si>
+    <t xml:space="preserve">QUOTED (eLearning code included, confirmed 3 Oct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Certified boat diving, 3 days / 6 dives (Mon-Wed) incl. boat fees, lunch, drinks, environmental fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED (Ras Mohammed and the Straits of Tiran, confirmed 3 Oct)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thursday morning boat, 2 dives, whole group, all included</t>
+  </si>
+  <si>
     <t xml:space="preserve">QUOTED</t>
   </si>
   <si>
-    <t xml:space="preserve">Certified boat diving, 3 days / 6 dives (Mon-Wed) incl. boat fees, lunch, drinks, environmental fee</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED (sites to confirm: Tiran, Ras Mohammed)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thursday morning boat, 2 dives, whole group, all included</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thistlegorm supplement (AOW + 20 logged dives)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED; add-on, not in the fee</t>
+    <t xml:space="preserve">Thistlegorm supplement (AOW + 20 logged dives), taken on the third boat day</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 3 Oct; add-on, not in the fee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Half-board supplement per person per night (dinner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 3 Oct 13:23; add-on so the beginner fee stays above certified</t>
   </si>
   <si>
     <t xml:space="preserve">Advanced Open Water, 2 days, all included</t>
@@ -171,10 +180,10 @@
     <t xml:space="preserve">Own spending guidance, not in the fee (no flights)</t>
   </si>
   <si>
-    <t xml:space="preserve">Airport transfers both ways, SSH to Naama Bay (about 15 minutes)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ASSUMED until RSDC prices it</t>
+    <t xml:space="preserve">Airport transfers both ways, SSH to Naama Bay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 3 Oct (approx., arranged by RSDC)</t>
   </si>
   <si>
     <t xml:space="preserve">Dive-accident cover, required</t>
@@ -252,6 +261,9 @@
     <t xml:space="preserve">Thistlegorm supplement (AOW + 20 dives)</t>
   </si>
   <si>
+    <t xml:space="preserve">Half board, 5 dinners</t>
+  </si>
+  <si>
     <t xml:space="preserve">GUIDANCE BUDGET WITHOUT FLIGHTS</t>
   </si>
   <si>
@@ -330,7 +342,7 @@
     <t xml:space="preserve">Covered?</t>
   </si>
   <si>
-    <t xml:space="preserve">Deposit and cancellation terms: RSDC will set them once the group size is known (QUOTED 3 Oct). Transfers priced on final numbers.</t>
+    <t xml:space="preserve">Deposit and cancellation terms: RSDC will set them once the group size is known (QUOTED 3 Oct). Space held to the end of October (QUOTED 3 Oct). RSDC is inside the Tao hotel on the Naama Bay promenade.</t>
   </si>
 </sst>
 </file>
@@ -738,7 +750,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="72"/>
@@ -868,7 +880,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
@@ -907,12 +919,12 @@
         <v>24</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>160</v>
@@ -921,60 +933,60 @@
         <v>24</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B15" s="7" t="n">
-        <v>395</v>
+        <v>15</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B16" s="7" t="n">
+        <v>395</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="7" t="n">
         <v>35</v>
       </c>
-      <c r="B17" s="5" t="n">
-        <v>4</v>
-      </c>
       <c r="C17" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B18" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>22</v>
@@ -982,172 +994,186 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B19" s="5" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>39</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="2"/>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2" t="s">
+      <c r="B20" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="7" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>43</v>
       </c>
+    </row>
+    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B22" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" s="7" t="n">
         <f aca="false">Inputs!$B$9*Inputs!$B$10*0.5</f>
         <v>175</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B23" s="7" t="n">
-        <f aca="false">Inputs!$B$16*4</f>
-        <v>140</v>
-      </c>
       <c r="C23" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" s="7" t="n">
+        <f aca="false">Inputs!$B$17*4</f>
+        <v>140</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>50</v>
-      </c>
+      <c r="A25" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B26" s="7" t="n">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B27" s="7" t="n">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>24</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B28" s="7" t="n">
         <v>30</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B29" s="7" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="5" t="n">
-        <v>5</v>
+        <v>60</v>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>25</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D30" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" s="7" t="n">
+        <v>62</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="7" t="n">
         <v>50</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D31" s="2" t="s">
-        <v>58</v>
+      <c r="D32" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1166,7 +1192,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="66"/>
@@ -1175,7 +1201,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1183,15 +1209,15 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B3" s="8" t="n">
         <f aca="false">Inputs!$B$11+Inputs!$B$13</f>
@@ -1204,20 +1230,20 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B4" s="8" t="n">
-        <f aca="false">Inputs!$B$16*Inputs!$B$18</f>
+        <f aca="false">Inputs!$B$17*Inputs!$B$19</f>
         <v>35</v>
       </c>
       <c r="C4" s="8" t="n">
-        <f aca="false">Inputs!$B$16*Inputs!$B$17</f>
+        <f aca="false">Inputs!$B$17*Inputs!$B$18</f>
         <v>140</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">Inputs!$B$9*Inputs!$B$10</f>
@@ -1230,20 +1256,20 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">(Inputs!$B$21+Inputs!$B$22+Inputs!$B$23)/(Inputs!$B$4-1)</f>
+        <f aca="false">(Inputs!$B$22+Inputs!$B$23+Inputs!$B$24)/(Inputs!$B$4-1)</f>
         <v>69.2105263157895</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">(Inputs!$B$21+Inputs!$B$22+Inputs!$B$23)/(Inputs!$B$4-1)</f>
+        <f aca="false">(Inputs!$B$22+Inputs!$B$23+Inputs!$B$24)/(Inputs!$B$4-1)</f>
         <v>69.2105263157895</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B7" s="9" t="n">
         <f aca="false">SUM(B3:B6)</f>
@@ -1256,7 +1282,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">ROUND(B7*Inputs!$B$7,0)</f>
@@ -1269,7 +1295,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B7+B8</f>
@@ -1282,7 +1308,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">CEILING(B9,50)</f>
@@ -1300,29 +1326,29 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C13" s="8" t="n">
-        <f aca="false">Inputs!$B$15</f>
+        <f aca="false">Inputs!$B$16</f>
         <v>395</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C14" s="8" t="n">
         <f aca="false">Inputs!$B$14</f>
@@ -1330,66 +1356,79 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
+      <c r="A15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">Inputs!$B$15*Inputs!$B$10</f>
+        <v>75</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">Inputs!$B$15*Inputs!$B$10</f>
+        <v>75</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="A16" s="2"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B17" s="9" t="n">
+      <c r="A17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="9" t="n">
         <f aca="false">B10</f>
         <v>1100</v>
       </c>
-      <c r="C17" s="9" t="n">
+      <c r="C18" s="9" t="n">
         <f aca="false">C10</f>
         <v>1050</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B18" s="8" t="n">
-        <f aca="false">Inputs!$B$25+Inputs!$B$26+Inputs!$B$27+(Inputs!$B$28+Inputs!$B$29)*Inputs!$B$30+Inputs!$B$31</f>
-        <v>469</v>
-      </c>
-      <c r="C18" s="8" t="n">
-        <f aca="false">Inputs!$B$25+Inputs!$B$26+Inputs!$B$27+(Inputs!$B$28+Inputs!$B$29)*Inputs!$B$30+Inputs!$B$31</f>
-        <v>469</v>
-      </c>
-    </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="9" t="n">
-        <f aca="false">B17+B18</f>
-        <v>1569</v>
-      </c>
-      <c r="C19" s="9" t="n">
-        <f aca="false">C17+C18</f>
-        <v>1519</v>
+      <c r="A19" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <f aca="false">Inputs!$B$26+Inputs!$B$27+Inputs!$B$28+(Inputs!$B$29+Inputs!$B$30)*Inputs!$B$31+Inputs!$B$32</f>
+        <v>454</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <f aca="false">Inputs!$B$26+Inputs!$B$27+Inputs!$B$28+(Inputs!$B$29+Inputs!$B$30)*Inputs!$B$31+Inputs!$B$32</f>
+        <v>454</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>74</v>
+        <v>83</v>
+      </c>
+      <c r="B20" s="9" t="n">
+        <f aca="false">B18+B19</f>
+        <v>1554</v>
       </c>
       <c r="C20" s="9" t="n">
-        <f aca="false">C19+C13+C14</f>
-        <v>2074</v>
+        <f aca="false">C18+C19</f>
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C21" s="9" t="n">
+        <f aca="false">C20+C13+C14</f>
+        <v>2059</v>
       </c>
     </row>
   </sheetData>
@@ -1417,7 +1456,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -1427,21 +1466,21 @@
     <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3"/>
       <c r="B2" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B3" s="10" t="n">
         <v>12</v>
@@ -1458,7 +1497,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B4" s="10" t="n">
         <f aca="false">B3-1</f>
@@ -1479,7 +1518,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B5" s="10" t="n">
         <f aca="false">ROUND(B4*Inputs!$B$6,0)</f>
@@ -1500,7 +1539,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B6" s="10" t="n">
         <f aca="false">B4-B5</f>
@@ -1521,28 +1560,28 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B7" s="10" t="n">
-        <f aca="false">INT(B4/Inputs!$B$19)</f>
+        <f aca="false">INT(B4/Inputs!$B$20)</f>
         <v>1</v>
       </c>
       <c r="C7" s="10" t="n">
-        <f aca="false">INT(C4/Inputs!$B$19)</f>
+        <f aca="false">INT(C4/Inputs!$B$20)</f>
         <v>1</v>
       </c>
       <c r="D7" s="10" t="n">
-        <f aca="false">INT(D4/Inputs!$B$19)</f>
+        <f aca="false">INT(D4/Inputs!$B$20)</f>
         <v>2</v>
       </c>
       <c r="E7" s="10" t="n">
-        <f aca="false">INT(E4/Inputs!$B$19)</f>
+        <f aca="false">INT(E4/Inputs!$B$20)</f>
         <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">B5*Fee!$B$10+B6*Fee!$C$10</f>
@@ -1563,7 +1602,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">B4*Inputs!$B$9*Inputs!$B$10</f>
@@ -1584,7 +1623,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">B5*(Inputs!$B$11+Inputs!$B$13)</f>
@@ -1605,7 +1644,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">B6*(Inputs!$B$12+Inputs!$B$13)</f>
@@ -1626,7 +1665,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">IF(B7&gt;=1,0,Inputs!$B$9*Inputs!$B$10+Inputs!$B$12+Inputs!$B$13)</f>
@@ -1647,7 +1686,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">-MAX(B7-1,0)*(Inputs!$B$9*Inputs!$B$10+Inputs!$B$12+Inputs!$B$13)</f>
@@ -1668,70 +1707,70 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B14" s="8" t="n">
-        <f aca="false">(B6+1)*Inputs!$B$16*Inputs!$B$17+B5*Inputs!$B$16*Inputs!$B$18</f>
+        <f aca="false">(B6+1)*Inputs!$B$17*Inputs!$B$18+B5*Inputs!$B$17*Inputs!$B$19</f>
         <v>1050</v>
       </c>
       <c r="C14" s="8" t="n">
-        <f aca="false">(C6+1)*Inputs!$B$16*Inputs!$B$17+C5*Inputs!$B$16*Inputs!$B$18</f>
+        <f aca="false">(C6+1)*Inputs!$B$17*Inputs!$B$18+C5*Inputs!$B$17*Inputs!$B$19</f>
         <v>1750</v>
       </c>
       <c r="D14" s="8" t="n">
-        <f aca="false">(D6+1)*Inputs!$B$16*Inputs!$B$17+D5*Inputs!$B$16*Inputs!$B$18</f>
+        <f aca="false">(D6+1)*Inputs!$B$17*Inputs!$B$18+D5*Inputs!$B$17*Inputs!$B$19</f>
         <v>2240</v>
       </c>
       <c r="E14" s="8" t="n">
-        <f aca="false">(E6+1)*Inputs!$B$16*Inputs!$B$17+E5*Inputs!$B$16*Inputs!$B$18</f>
+        <f aca="false">(E6+1)*Inputs!$B$17*Inputs!$B$18+E5*Inputs!$B$17*Inputs!$B$19</f>
         <v>2625</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="2" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B15" s="8" t="n">
-        <f aca="false">IF(MOD(B3,2)=1,Inputs!$B$22,0)</f>
+        <f aca="false">IF(MOD(B3,2)=1,Inputs!$B$23,0)</f>
         <v>0</v>
       </c>
       <c r="C15" s="8" t="n">
-        <f aca="false">IF(MOD(C3,2)=1,Inputs!$B$22,0)</f>
+        <f aca="false">IF(MOD(C3,2)=1,Inputs!$B$23,0)</f>
         <v>0</v>
       </c>
       <c r="D15" s="8" t="n">
-        <f aca="false">IF(MOD(D3,2)=1,Inputs!$B$22,0)</f>
+        <f aca="false">IF(MOD(D3,2)=1,Inputs!$B$23,0)</f>
         <v>175</v>
       </c>
       <c r="E15" s="8" t="n">
-        <f aca="false">IF(MOD(E3,2)=1,Inputs!$B$22,0)</f>
+        <f aca="false">IF(MOD(E3,2)=1,Inputs!$B$23,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B16" s="8" t="n">
-        <f aca="false">Inputs!$B$21</f>
+        <f aca="false">Inputs!$B$22</f>
         <v>1000</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">Inputs!$B$21</f>
+        <f aca="false">Inputs!$B$22</f>
         <v>1000</v>
       </c>
       <c r="D16" s="8" t="n">
-        <f aca="false">Inputs!$B$21</f>
+        <f aca="false">Inputs!$B$22</f>
         <v>1000</v>
       </c>
       <c r="E16" s="8" t="n">
-        <f aca="false">Inputs!$B$21</f>
+        <f aca="false">Inputs!$B$22</f>
         <v>1000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">B9+B10+B11+B12+B13+B14+B15+B16</f>
@@ -1752,7 +1791,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">B8-B17</f>
@@ -1773,7 +1812,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B19" s="11" t="str">
         <f aca="false">IF(B18&gt;=0,"yes","NO")</f>
@@ -1792,9 +1831,9 @@
         <v>yes</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>

</xml_diff>